<commit_message>
celldata auch einzeln abrufbar, kommentierung
</commit_message>
<xml_diff>
--- a/Core/Inc/ds_lookup_01_05.xlsx
+++ b/Core/Inc/ds_lookup_01_05.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\res\STM32CubeIDE\workspace_1.12.0\bms-blk\Core\Inc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A389C624-EE41-4D49-92BF-082D87E92434}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{834B7DFB-CE4A-4ABF-AB6E-CFD25EAAD109}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="41670" yWindow="2100" windowWidth="28800" windowHeight="15435" activeTab="1" xr2:uid="{D4473AF3-D1EF-406D-B595-001F811C9F16}"/>
+    <workbookView xWindow="7350" yWindow="345" windowWidth="28800" windowHeight="19770" xr2:uid="{D4473AF3-D1EF-406D-B595-001F811C9F16}"/>
   </bookViews>
   <sheets>
-    <sheet name="BAT1_BLK01 (2)" sheetId="4" r:id="rId1"/>
-    <sheet name="BAT1_BRD_05" sheetId="3" r:id="rId2"/>
-    <sheet name="BAT1_BLK04" sheetId="1" r:id="rId3"/>
-    <sheet name="BAT1_BLK05" sheetId="2" r:id="rId4"/>
+    <sheet name="BAT2_BRD_07" sheetId="5" r:id="rId1"/>
+    <sheet name="BAT1_BLK01 (2)" sheetId="4" r:id="rId2"/>
+    <sheet name="BAT1_BRD_05" sheetId="3" r:id="rId3"/>
+    <sheet name="BAT1_BLK04" sheetId="1" r:id="rId4"/>
+    <sheet name="BAT1_BLK05" sheetId="2" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1245" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1655" uniqueCount="167">
   <si>
     <t>0x28</t>
   </si>
@@ -469,16 +470,91 @@
   </si>
   <si>
     <t>onboard_temp</t>
+  </si>
+  <si>
+    <t>0x39</t>
+  </si>
+  <si>
+    <t>0x56</t>
+  </si>
+  <si>
+    <t>0xD4</t>
+  </si>
+  <si>
+    <t>0xB0</t>
+  </si>
+  <si>
+    <t>0x67</t>
+  </si>
+  <si>
+    <t>0x06</t>
+  </si>
+  <si>
+    <t>0x91</t>
+  </si>
+  <si>
+    <t>0x12</t>
+  </si>
+  <si>
+    <t>0x0A</t>
+  </si>
+  <si>
+    <t>0xEB</t>
+  </si>
+  <si>
+    <t>0xD1</t>
+  </si>
+  <si>
+    <t>0x7F</t>
+  </si>
+  <si>
+    <t>0x19</t>
+  </si>
+  <si>
+    <t>0xED</t>
+  </si>
+  <si>
+    <t>0xB1</t>
+  </si>
+  <si>
+    <t>0x5F</t>
+  </si>
+  <si>
+    <t>0xF3</t>
+  </si>
+  <si>
+    <t>0x48</t>
+  </si>
+  <si>
+    <t>0x43</t>
+  </si>
+  <si>
+    <t>0x8F</t>
+  </si>
+  <si>
+    <t>0x1F</t>
+  </si>
+  <si>
+    <t>0xF7</t>
+  </si>
+  <si>
+    <t>0x13</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -819,6 +895,1449 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35699E4F-4303-4953-AE64-D09B1A493B0E}">
+  <dimension ref="A4:T27"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="3.7109375" customWidth="1"/>
+    <col min="3" max="3" width="2.85546875" customWidth="1"/>
+    <col min="4" max="4" width="7" customWidth="1"/>
+    <col min="5" max="5" width="3.28515625" customWidth="1"/>
+    <col min="6" max="6" width="7.140625" customWidth="1"/>
+    <col min="7" max="7" width="2.85546875" customWidth="1"/>
+    <col min="8" max="8" width="6.28515625" customWidth="1"/>
+    <col min="9" max="9" width="3" customWidth="1"/>
+    <col min="10" max="10" width="6" customWidth="1"/>
+    <col min="11" max="11" width="2.7109375" customWidth="1"/>
+    <col min="12" max="12" width="5.5703125" customWidth="1"/>
+    <col min="13" max="13" width="2.140625" customWidth="1"/>
+    <col min="14" max="14" width="6.7109375" customWidth="1"/>
+    <col min="15" max="15" width="2.85546875" customWidth="1"/>
+    <col min="16" max="16" width="6.140625" customWidth="1"/>
+    <col min="17" max="17" width="2.42578125" customWidth="1"/>
+    <col min="18" max="18" width="7" customWidth="1"/>
+    <col min="19" max="19" width="3.140625" customWidth="1"/>
+    <col min="20" max="20" width="2.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>0</v>
+      </c>
+      <c r="C4" t="s">
+        <v>71</v>
+      </c>
+      <c r="D4" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" t="s">
+        <v>70</v>
+      </c>
+      <c r="F4" t="s">
+        <v>1</v>
+      </c>
+      <c r="G4" t="s">
+        <v>70</v>
+      </c>
+      <c r="H4" t="s">
+        <v>2</v>
+      </c>
+      <c r="I4" t="s">
+        <v>70</v>
+      </c>
+      <c r="J4" t="s">
+        <v>3</v>
+      </c>
+      <c r="K4" t="s">
+        <v>70</v>
+      </c>
+      <c r="M4" t="s">
+        <v>70</v>
+      </c>
+      <c r="O4" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>70</v>
+      </c>
+      <c r="S4" t="s">
+        <v>72</v>
+      </c>
+      <c r="T4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>1</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6" t="s">
+        <v>71</v>
+      </c>
+      <c r="D6" t="s">
+        <v>0</v>
+      </c>
+      <c r="E6" t="s">
+        <v>70</v>
+      </c>
+      <c r="F6" t="s">
+        <v>1</v>
+      </c>
+      <c r="G6" t="s">
+        <v>70</v>
+      </c>
+      <c r="H6" t="s">
+        <v>2</v>
+      </c>
+      <c r="I6" t="s">
+        <v>70</v>
+      </c>
+      <c r="J6" t="s">
+        <v>3</v>
+      </c>
+      <c r="K6" t="s">
+        <v>70</v>
+      </c>
+      <c r="L6" t="s">
+        <v>4</v>
+      </c>
+      <c r="M6" t="s">
+        <v>70</v>
+      </c>
+      <c r="N6" t="s">
+        <v>5</v>
+      </c>
+      <c r="O6" t="s">
+        <v>70</v>
+      </c>
+      <c r="P6" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>70</v>
+      </c>
+      <c r="R6" t="s">
+        <v>48</v>
+      </c>
+      <c r="S6" t="s">
+        <v>72</v>
+      </c>
+      <c r="T6" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>2</v>
+      </c>
+      <c r="B7">
+        <v>20</v>
+      </c>
+      <c r="C7" t="s">
+        <v>71</v>
+      </c>
+      <c r="D7" t="s">
+        <v>0</v>
+      </c>
+      <c r="E7" t="s">
+        <v>70</v>
+      </c>
+      <c r="F7" t="s">
+        <v>1</v>
+      </c>
+      <c r="G7" t="s">
+        <v>70</v>
+      </c>
+      <c r="H7" t="s">
+        <v>2</v>
+      </c>
+      <c r="I7" t="s">
+        <v>70</v>
+      </c>
+      <c r="J7" t="s">
+        <v>3</v>
+      </c>
+      <c r="K7" t="s">
+        <v>70</v>
+      </c>
+      <c r="L7" t="s">
+        <v>12</v>
+      </c>
+      <c r="M7" t="s">
+        <v>70</v>
+      </c>
+      <c r="N7" t="s">
+        <v>30</v>
+      </c>
+      <c r="O7" t="s">
+        <v>70</v>
+      </c>
+      <c r="P7" t="s">
+        <v>147</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>70</v>
+      </c>
+      <c r="R7" t="s">
+        <v>146</v>
+      </c>
+      <c r="S7" t="s">
+        <v>72</v>
+      </c>
+      <c r="T7" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>3</v>
+      </c>
+      <c r="B8">
+        <v>15</v>
+      </c>
+      <c r="C8" t="s">
+        <v>71</v>
+      </c>
+      <c r="D8" t="s">
+        <v>0</v>
+      </c>
+      <c r="E8" t="s">
+        <v>70</v>
+      </c>
+      <c r="F8" t="s">
+        <v>1</v>
+      </c>
+      <c r="G8" t="s">
+        <v>70</v>
+      </c>
+      <c r="H8" t="s">
+        <v>2</v>
+      </c>
+      <c r="I8" t="s">
+        <v>70</v>
+      </c>
+      <c r="J8" t="s">
+        <v>3</v>
+      </c>
+      <c r="K8" t="s">
+        <v>70</v>
+      </c>
+      <c r="L8" t="s">
+        <v>8</v>
+      </c>
+      <c r="M8" t="s">
+        <v>70</v>
+      </c>
+      <c r="N8" t="s">
+        <v>148</v>
+      </c>
+      <c r="O8" t="s">
+        <v>70</v>
+      </c>
+      <c r="P8" t="s">
+        <v>149</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>70</v>
+      </c>
+      <c r="R8" t="s">
+        <v>102</v>
+      </c>
+      <c r="S8" t="s">
+        <v>72</v>
+      </c>
+      <c r="T8" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>4</v>
+      </c>
+      <c r="B9">
+        <v>16</v>
+      </c>
+      <c r="C9" t="s">
+        <v>71</v>
+      </c>
+      <c r="D9" t="s">
+        <v>0</v>
+      </c>
+      <c r="E9" t="s">
+        <v>70</v>
+      </c>
+      <c r="F9" t="s">
+        <v>1</v>
+      </c>
+      <c r="G9" t="s">
+        <v>70</v>
+      </c>
+      <c r="H9" t="s">
+        <v>2</v>
+      </c>
+      <c r="I9" t="s">
+        <v>70</v>
+      </c>
+      <c r="J9" t="s">
+        <v>3</v>
+      </c>
+      <c r="K9" t="s">
+        <v>70</v>
+      </c>
+      <c r="L9" t="s">
+        <v>8</v>
+      </c>
+      <c r="M9" t="s">
+        <v>70</v>
+      </c>
+      <c r="N9" t="s">
+        <v>121</v>
+      </c>
+      <c r="O9" t="s">
+        <v>70</v>
+      </c>
+      <c r="P9" t="s">
+        <v>145</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>70</v>
+      </c>
+      <c r="R9" t="s">
+        <v>63</v>
+      </c>
+      <c r="S9" t="s">
+        <v>72</v>
+      </c>
+      <c r="T9" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>5</v>
+      </c>
+      <c r="B10">
+        <v>12</v>
+      </c>
+      <c r="C10" t="s">
+        <v>71</v>
+      </c>
+      <c r="D10" t="s">
+        <v>0</v>
+      </c>
+      <c r="E10" t="s">
+        <v>70</v>
+      </c>
+      <c r="F10" t="s">
+        <v>1</v>
+      </c>
+      <c r="G10" t="s">
+        <v>70</v>
+      </c>
+      <c r="H10" t="s">
+        <v>2</v>
+      </c>
+      <c r="I10" t="s">
+        <v>70</v>
+      </c>
+      <c r="J10" t="s">
+        <v>3</v>
+      </c>
+      <c r="K10" t="s">
+        <v>70</v>
+      </c>
+      <c r="L10" t="s">
+        <v>4</v>
+      </c>
+      <c r="M10" t="s">
+        <v>70</v>
+      </c>
+      <c r="N10" t="s">
+        <v>137</v>
+      </c>
+      <c r="O10" t="s">
+        <v>70</v>
+      </c>
+      <c r="P10" t="s">
+        <v>117</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>70</v>
+      </c>
+      <c r="R10" t="s">
+        <v>85</v>
+      </c>
+      <c r="S10" t="s">
+        <v>72</v>
+      </c>
+      <c r="T10" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>6</v>
+      </c>
+      <c r="B11">
+        <v>14</v>
+      </c>
+      <c r="C11" t="s">
+        <v>71</v>
+      </c>
+      <c r="D11" t="s">
+        <v>0</v>
+      </c>
+      <c r="E11" t="s">
+        <v>70</v>
+      </c>
+      <c r="F11" t="s">
+        <v>1</v>
+      </c>
+      <c r="G11" t="s">
+        <v>70</v>
+      </c>
+      <c r="H11" t="s">
+        <v>2</v>
+      </c>
+      <c r="I11" t="s">
+        <v>70</v>
+      </c>
+      <c r="J11" t="s">
+        <v>3</v>
+      </c>
+      <c r="K11" t="s">
+        <v>70</v>
+      </c>
+      <c r="L11" t="s">
+        <v>4</v>
+      </c>
+      <c r="M11" t="s">
+        <v>70</v>
+      </c>
+      <c r="N11" t="s">
+        <v>45</v>
+      </c>
+      <c r="O11" t="s">
+        <v>70</v>
+      </c>
+      <c r="P11" t="s">
+        <v>150</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>70</v>
+      </c>
+      <c r="R11" t="s">
+        <v>151</v>
+      </c>
+      <c r="S11" t="s">
+        <v>72</v>
+      </c>
+      <c r="T11" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>7</v>
+      </c>
+      <c r="B12">
+        <v>22</v>
+      </c>
+      <c r="C12" t="s">
+        <v>71</v>
+      </c>
+      <c r="D12" t="s">
+        <v>0</v>
+      </c>
+      <c r="E12" t="s">
+        <v>70</v>
+      </c>
+      <c r="F12" t="s">
+        <v>1</v>
+      </c>
+      <c r="G12" t="s">
+        <v>70</v>
+      </c>
+      <c r="H12" t="s">
+        <v>2</v>
+      </c>
+      <c r="I12" t="s">
+        <v>70</v>
+      </c>
+      <c r="J12" t="s">
+        <v>3</v>
+      </c>
+      <c r="K12" t="s">
+        <v>70</v>
+      </c>
+      <c r="L12" t="s">
+        <v>12</v>
+      </c>
+      <c r="M12" t="s">
+        <v>70</v>
+      </c>
+      <c r="N12" t="s">
+        <v>149</v>
+      </c>
+      <c r="O12" t="s">
+        <v>70</v>
+      </c>
+      <c r="P12" t="s">
+        <v>91</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>70</v>
+      </c>
+      <c r="R12" t="s">
+        <v>152</v>
+      </c>
+      <c r="S12" t="s">
+        <v>72</v>
+      </c>
+      <c r="T12" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>8</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>71</v>
+      </c>
+      <c r="D13" t="s">
+        <v>0</v>
+      </c>
+      <c r="E13" t="s">
+        <v>70</v>
+      </c>
+      <c r="F13" t="s">
+        <v>1</v>
+      </c>
+      <c r="G13" t="s">
+        <v>70</v>
+      </c>
+      <c r="H13" t="s">
+        <v>2</v>
+      </c>
+      <c r="I13" t="s">
+        <v>70</v>
+      </c>
+      <c r="J13" t="s">
+        <v>3</v>
+      </c>
+      <c r="K13" t="s">
+        <v>70</v>
+      </c>
+      <c r="L13" t="s">
+        <v>4</v>
+      </c>
+      <c r="M13" t="s">
+        <v>70</v>
+      </c>
+      <c r="N13" t="s">
+        <v>153</v>
+      </c>
+      <c r="O13" t="s">
+        <v>70</v>
+      </c>
+      <c r="P13" t="s">
+        <v>154</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>70</v>
+      </c>
+      <c r="R13" t="s">
+        <v>26</v>
+      </c>
+      <c r="S13" t="s">
+        <v>72</v>
+      </c>
+      <c r="T13" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>9</v>
+      </c>
+      <c r="B14">
+        <v>9</v>
+      </c>
+      <c r="C14" t="s">
+        <v>71</v>
+      </c>
+      <c r="D14" t="s">
+        <v>0</v>
+      </c>
+      <c r="E14" t="s">
+        <v>70</v>
+      </c>
+      <c r="F14" t="s">
+        <v>1</v>
+      </c>
+      <c r="G14" t="s">
+        <v>70</v>
+      </c>
+      <c r="H14" t="s">
+        <v>2</v>
+      </c>
+      <c r="I14" t="s">
+        <v>70</v>
+      </c>
+      <c r="J14" t="s">
+        <v>3</v>
+      </c>
+      <c r="K14" t="s">
+        <v>70</v>
+      </c>
+      <c r="L14" t="s">
+        <v>4</v>
+      </c>
+      <c r="M14" t="s">
+        <v>70</v>
+      </c>
+      <c r="N14" t="s">
+        <v>54</v>
+      </c>
+      <c r="O14" t="s">
+        <v>70</v>
+      </c>
+      <c r="P14" t="s">
+        <v>140</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>70</v>
+      </c>
+      <c r="R14" t="s">
+        <v>73</v>
+      </c>
+      <c r="S14" t="s">
+        <v>72</v>
+      </c>
+      <c r="T14" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>10</v>
+      </c>
+      <c r="B15">
+        <v>18</v>
+      </c>
+      <c r="C15" t="s">
+        <v>71</v>
+      </c>
+      <c r="D15" t="s">
+        <v>0</v>
+      </c>
+      <c r="E15" t="s">
+        <v>70</v>
+      </c>
+      <c r="F15" t="s">
+        <v>1</v>
+      </c>
+      <c r="G15" t="s">
+        <v>70</v>
+      </c>
+      <c r="H15" t="s">
+        <v>2</v>
+      </c>
+      <c r="I15" t="s">
+        <v>70</v>
+      </c>
+      <c r="J15" t="s">
+        <v>3</v>
+      </c>
+      <c r="K15" t="s">
+        <v>70</v>
+      </c>
+      <c r="L15" t="s">
+        <v>12</v>
+      </c>
+      <c r="M15" t="s">
+        <v>70</v>
+      </c>
+      <c r="N15" t="s">
+        <v>116</v>
+      </c>
+      <c r="O15" t="s">
+        <v>70</v>
+      </c>
+      <c r="P15" t="s">
+        <v>155</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>70</v>
+      </c>
+      <c r="R15" t="s">
+        <v>156</v>
+      </c>
+      <c r="S15" t="s">
+        <v>72</v>
+      </c>
+      <c r="T15" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>11</v>
+      </c>
+      <c r="B16">
+        <v>21</v>
+      </c>
+      <c r="C16" t="s">
+        <v>71</v>
+      </c>
+      <c r="D16" t="s">
+        <v>0</v>
+      </c>
+      <c r="E16" t="s">
+        <v>70</v>
+      </c>
+      <c r="F16" t="s">
+        <v>1</v>
+      </c>
+      <c r="G16" t="s">
+        <v>70</v>
+      </c>
+      <c r="H16" t="s">
+        <v>2</v>
+      </c>
+      <c r="I16" t="s">
+        <v>70</v>
+      </c>
+      <c r="J16" t="s">
+        <v>3</v>
+      </c>
+      <c r="K16" t="s">
+        <v>70</v>
+      </c>
+      <c r="L16" t="s">
+        <v>12</v>
+      </c>
+      <c r="M16" t="s">
+        <v>70</v>
+      </c>
+      <c r="N16" t="s">
+        <v>149</v>
+      </c>
+      <c r="O16" t="s">
+        <v>70</v>
+      </c>
+      <c r="P16" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>70</v>
+      </c>
+      <c r="R16" t="s">
+        <v>28</v>
+      </c>
+      <c r="S16" t="s">
+        <v>72</v>
+      </c>
+      <c r="T16" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>12</v>
+      </c>
+      <c r="B17">
+        <v>5</v>
+      </c>
+      <c r="C17" t="s">
+        <v>71</v>
+      </c>
+      <c r="D17" t="s">
+        <v>0</v>
+      </c>
+      <c r="E17" t="s">
+        <v>70</v>
+      </c>
+      <c r="F17" t="s">
+        <v>1</v>
+      </c>
+      <c r="G17" t="s">
+        <v>70</v>
+      </c>
+      <c r="H17" t="s">
+        <v>2</v>
+      </c>
+      <c r="I17" t="s">
+        <v>70</v>
+      </c>
+      <c r="J17" t="s">
+        <v>3</v>
+      </c>
+      <c r="K17" t="s">
+        <v>70</v>
+      </c>
+      <c r="L17" t="s">
+        <v>4</v>
+      </c>
+      <c r="M17" t="s">
+        <v>70</v>
+      </c>
+      <c r="N17" t="s">
+        <v>49</v>
+      </c>
+      <c r="O17" t="s">
+        <v>70</v>
+      </c>
+      <c r="P17" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>70</v>
+      </c>
+      <c r="R17" t="s">
+        <v>157</v>
+      </c>
+      <c r="S17" t="s">
+        <v>72</v>
+      </c>
+      <c r="T17" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>13</v>
+      </c>
+      <c r="B18">
+        <v>19</v>
+      </c>
+      <c r="C18" t="s">
+        <v>71</v>
+      </c>
+      <c r="D18" t="s">
+        <v>0</v>
+      </c>
+      <c r="E18" t="s">
+        <v>70</v>
+      </c>
+      <c r="F18" t="s">
+        <v>1</v>
+      </c>
+      <c r="G18" t="s">
+        <v>70</v>
+      </c>
+      <c r="H18" t="s">
+        <v>2</v>
+      </c>
+      <c r="I18" t="s">
+        <v>70</v>
+      </c>
+      <c r="J18" t="s">
+        <v>3</v>
+      </c>
+      <c r="K18" t="s">
+        <v>70</v>
+      </c>
+      <c r="L18" t="s">
+        <v>12</v>
+      </c>
+      <c r="M18" t="s">
+        <v>70</v>
+      </c>
+      <c r="N18" t="s">
+        <v>49</v>
+      </c>
+      <c r="O18" t="s">
+        <v>70</v>
+      </c>
+      <c r="P18" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>70</v>
+      </c>
+      <c r="R18" t="s">
+        <v>131</v>
+      </c>
+      <c r="S18" t="s">
+        <v>72</v>
+      </c>
+      <c r="T18" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>14</v>
+      </c>
+      <c r="B19">
+        <v>1</v>
+      </c>
+      <c r="C19" t="s">
+        <v>71</v>
+      </c>
+      <c r="D19" t="s">
+        <v>0</v>
+      </c>
+      <c r="E19" t="s">
+        <v>70</v>
+      </c>
+      <c r="F19" t="s">
+        <v>1</v>
+      </c>
+      <c r="G19" t="s">
+        <v>70</v>
+      </c>
+      <c r="H19" t="s">
+        <v>2</v>
+      </c>
+      <c r="I19" t="s">
+        <v>70</v>
+      </c>
+      <c r="J19" t="s">
+        <v>3</v>
+      </c>
+      <c r="K19" t="s">
+        <v>70</v>
+      </c>
+      <c r="L19" t="s">
+        <v>4</v>
+      </c>
+      <c r="M19" t="s">
+        <v>70</v>
+      </c>
+      <c r="N19" t="s">
+        <v>5</v>
+      </c>
+      <c r="O19" t="s">
+        <v>70</v>
+      </c>
+      <c r="P19" t="s">
+        <v>158</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>70</v>
+      </c>
+      <c r="R19" t="s">
+        <v>159</v>
+      </c>
+      <c r="S19" t="s">
+        <v>72</v>
+      </c>
+      <c r="T19" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>15</v>
+      </c>
+      <c r="B20">
+        <v>8</v>
+      </c>
+      <c r="C20" t="s">
+        <v>71</v>
+      </c>
+      <c r="D20" t="s">
+        <v>0</v>
+      </c>
+      <c r="E20" t="s">
+        <v>70</v>
+      </c>
+      <c r="F20" t="s">
+        <v>1</v>
+      </c>
+      <c r="G20" t="s">
+        <v>70</v>
+      </c>
+      <c r="H20" t="s">
+        <v>2</v>
+      </c>
+      <c r="I20" t="s">
+        <v>70</v>
+      </c>
+      <c r="J20" t="s">
+        <v>3</v>
+      </c>
+      <c r="K20" t="s">
+        <v>70</v>
+      </c>
+      <c r="L20" t="s">
+        <v>4</v>
+      </c>
+      <c r="M20" t="s">
+        <v>70</v>
+      </c>
+      <c r="N20" t="s">
+        <v>38</v>
+      </c>
+      <c r="O20" t="s">
+        <v>70</v>
+      </c>
+      <c r="P20" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>70</v>
+      </c>
+      <c r="R20" t="s">
+        <v>160</v>
+      </c>
+      <c r="S20" t="s">
+        <v>72</v>
+      </c>
+      <c r="T20" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>16</v>
+      </c>
+      <c r="B21">
+        <v>6</v>
+      </c>
+      <c r="C21" t="s">
+        <v>71</v>
+      </c>
+      <c r="D21" t="s">
+        <v>0</v>
+      </c>
+      <c r="E21" t="s">
+        <v>70</v>
+      </c>
+      <c r="F21" t="s">
+        <v>1</v>
+      </c>
+      <c r="G21" t="s">
+        <v>70</v>
+      </c>
+      <c r="H21" t="s">
+        <v>2</v>
+      </c>
+      <c r="I21" t="s">
+        <v>70</v>
+      </c>
+      <c r="J21" t="s">
+        <v>3</v>
+      </c>
+      <c r="K21" t="s">
+        <v>70</v>
+      </c>
+      <c r="L21" t="s">
+        <v>4</v>
+      </c>
+      <c r="M21" t="s">
+        <v>70</v>
+      </c>
+      <c r="N21" t="s">
+        <v>90</v>
+      </c>
+      <c r="O21" t="s">
+        <v>70</v>
+      </c>
+      <c r="P21" t="s">
+        <v>89</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>70</v>
+      </c>
+      <c r="R21" t="s">
+        <v>26</v>
+      </c>
+      <c r="S21" t="s">
+        <v>72</v>
+      </c>
+      <c r="T21" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>17</v>
+      </c>
+      <c r="B22">
+        <v>13</v>
+      </c>
+      <c r="C22" t="s">
+        <v>71</v>
+      </c>
+      <c r="D22" t="s">
+        <v>0</v>
+      </c>
+      <c r="E22" t="s">
+        <v>70</v>
+      </c>
+      <c r="F22" t="s">
+        <v>1</v>
+      </c>
+      <c r="G22" t="s">
+        <v>70</v>
+      </c>
+      <c r="H22" t="s">
+        <v>2</v>
+      </c>
+      <c r="I22" t="s">
+        <v>70</v>
+      </c>
+      <c r="J22" t="s">
+        <v>3</v>
+      </c>
+      <c r="K22" t="s">
+        <v>70</v>
+      </c>
+      <c r="L22" t="s">
+        <v>4</v>
+      </c>
+      <c r="M22" t="s">
+        <v>70</v>
+      </c>
+      <c r="N22" t="s">
+        <v>161</v>
+      </c>
+      <c r="O22" t="s">
+        <v>70</v>
+      </c>
+      <c r="P22" t="s">
+        <v>90</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>70</v>
+      </c>
+      <c r="R22" t="s">
+        <v>17</v>
+      </c>
+      <c r="S22" t="s">
+        <v>72</v>
+      </c>
+      <c r="T22" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>18</v>
+      </c>
+      <c r="B23">
+        <v>4</v>
+      </c>
+      <c r="C23" t="s">
+        <v>71</v>
+      </c>
+      <c r="D23" t="s">
+        <v>0</v>
+      </c>
+      <c r="E23" t="s">
+        <v>70</v>
+      </c>
+      <c r="F23" t="s">
+        <v>1</v>
+      </c>
+      <c r="G23" t="s">
+        <v>70</v>
+      </c>
+      <c r="H23" t="s">
+        <v>2</v>
+      </c>
+      <c r="I23" t="s">
+        <v>70</v>
+      </c>
+      <c r="J23" t="s">
+        <v>3</v>
+      </c>
+      <c r="K23" t="s">
+        <v>70</v>
+      </c>
+      <c r="L23" t="s">
+        <v>4</v>
+      </c>
+      <c r="M23" t="s">
+        <v>70</v>
+      </c>
+      <c r="N23" t="s">
+        <v>162</v>
+      </c>
+      <c r="O23" t="s">
+        <v>70</v>
+      </c>
+      <c r="P23" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>70</v>
+      </c>
+      <c r="R23" t="s">
+        <v>163</v>
+      </c>
+      <c r="S23" t="s">
+        <v>72</v>
+      </c>
+      <c r="T23" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>19</v>
+      </c>
+      <c r="B24">
+        <v>10</v>
+      </c>
+      <c r="C24" t="s">
+        <v>71</v>
+      </c>
+      <c r="D24" t="s">
+        <v>0</v>
+      </c>
+      <c r="E24" t="s">
+        <v>70</v>
+      </c>
+      <c r="F24" t="s">
+        <v>1</v>
+      </c>
+      <c r="G24" t="s">
+        <v>70</v>
+      </c>
+      <c r="H24" t="s">
+        <v>2</v>
+      </c>
+      <c r="I24" t="s">
+        <v>70</v>
+      </c>
+      <c r="J24" t="s">
+        <v>3</v>
+      </c>
+      <c r="K24" t="s">
+        <v>70</v>
+      </c>
+      <c r="L24" t="s">
+        <v>4</v>
+      </c>
+      <c r="M24" t="s">
+        <v>70</v>
+      </c>
+      <c r="N24" t="s">
+        <v>107</v>
+      </c>
+      <c r="O24" t="s">
+        <v>70</v>
+      </c>
+      <c r="P24" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>70</v>
+      </c>
+      <c r="R24" t="s">
+        <v>3</v>
+      </c>
+      <c r="S24" t="s">
+        <v>72</v>
+      </c>
+      <c r="T24" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>20</v>
+      </c>
+      <c r="B25">
+        <v>17</v>
+      </c>
+      <c r="C25" t="s">
+        <v>71</v>
+      </c>
+      <c r="D25" t="s">
+        <v>0</v>
+      </c>
+      <c r="E25" t="s">
+        <v>70</v>
+      </c>
+      <c r="F25" t="s">
+        <v>1</v>
+      </c>
+      <c r="G25" t="s">
+        <v>70</v>
+      </c>
+      <c r="H25" t="s">
+        <v>2</v>
+      </c>
+      <c r="I25" t="s">
+        <v>70</v>
+      </c>
+      <c r="J25" t="s">
+        <v>3</v>
+      </c>
+      <c r="K25" t="s">
+        <v>70</v>
+      </c>
+      <c r="L25" t="s">
+        <v>15</v>
+      </c>
+      <c r="M25" t="s">
+        <v>70</v>
+      </c>
+      <c r="N25" t="s">
+        <v>164</v>
+      </c>
+      <c r="O25" t="s">
+        <v>70</v>
+      </c>
+      <c r="P25" t="s">
+        <v>165</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>70</v>
+      </c>
+      <c r="R25" t="s">
+        <v>121</v>
+      </c>
+      <c r="S25" t="s">
+        <v>72</v>
+      </c>
+      <c r="T25" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>21</v>
+      </c>
+      <c r="B26">
+        <v>11</v>
+      </c>
+      <c r="C26" t="s">
+        <v>71</v>
+      </c>
+      <c r="D26" t="s">
+        <v>0</v>
+      </c>
+      <c r="E26" t="s">
+        <v>70</v>
+      </c>
+      <c r="F26" t="s">
+        <v>1</v>
+      </c>
+      <c r="G26" t="s">
+        <v>70</v>
+      </c>
+      <c r="H26" t="s">
+        <v>2</v>
+      </c>
+      <c r="I26" t="s">
+        <v>70</v>
+      </c>
+      <c r="J26" t="s">
+        <v>3</v>
+      </c>
+      <c r="K26" t="s">
+        <v>70</v>
+      </c>
+      <c r="L26" t="s">
+        <v>4</v>
+      </c>
+      <c r="M26" t="s">
+        <v>70</v>
+      </c>
+      <c r="N26" t="s">
+        <v>129</v>
+      </c>
+      <c r="O26" t="s">
+        <v>70</v>
+      </c>
+      <c r="P26" t="s">
+        <v>166</v>
+      </c>
+      <c r="Q26" t="s">
+        <v>70</v>
+      </c>
+      <c r="R26" t="s">
+        <v>11</v>
+      </c>
+      <c r="S26" t="s">
+        <v>72</v>
+      </c>
+      <c r="T26" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>22</v>
+      </c>
+      <c r="B27">
+        <v>7</v>
+      </c>
+      <c r="C27" t="s">
+        <v>71</v>
+      </c>
+      <c r="D27" t="s">
+        <v>0</v>
+      </c>
+      <c r="E27" t="s">
+        <v>70</v>
+      </c>
+      <c r="F27" t="s">
+        <v>1</v>
+      </c>
+      <c r="G27" t="s">
+        <v>70</v>
+      </c>
+      <c r="H27" t="s">
+        <v>2</v>
+      </c>
+      <c r="I27" t="s">
+        <v>70</v>
+      </c>
+      <c r="J27" t="s">
+        <v>3</v>
+      </c>
+      <c r="K27" t="s">
+        <v>70</v>
+      </c>
+      <c r="L27" t="s">
+        <v>4</v>
+      </c>
+      <c r="M27" t="s">
+        <v>70</v>
+      </c>
+      <c r="N27" t="s">
+        <v>144</v>
+      </c>
+      <c r="O27" t="s">
+        <v>70</v>
+      </c>
+      <c r="P27" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q27" t="s">
+        <v>70</v>
+      </c>
+      <c r="R27" t="s">
+        <v>145</v>
+      </c>
+      <c r="S27" t="s">
+        <v>72</v>
+      </c>
+      <c r="T27" t="s">
+        <v>70</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56ACEB68-459E-4B8A-91B6-10D646747FBA}">
   <dimension ref="A4:V27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2260,7 +3779,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5CFFDA2-9D8B-4069-AA63-0D049CFF3673}">
   <dimension ref="A4:V4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2353,7 +3872,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8F420D1-D23F-4201-85FC-61080ADED44B}">
   <dimension ref="A4:T26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3741,7 +5260,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7B0B922-F444-49EF-A1D0-D03B87F5C0C4}">
   <dimension ref="A4:V26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>